<commit_message>
Added new notebooks and new events.
</commit_message>
<xml_diff>
--- a/Worcester Chorus current members.xlsx
+++ b/Worcester Chorus current members.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10402"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/antho/Documents/WPI-MW/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adrie\OneDrive\Desktop\MW\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A84578ED-064F-0246-979C-22F88A908679}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{D8976AD1-8FB8-4A80-92AC-66A7817CC3F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" xr2:uid="{CC2CE05C-E54E-4EE9-92C1-3AF990D82AF0}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CC2CE05C-E54E-4EE9-92C1-3AF990D82AF0}"/>
   </bookViews>
   <sheets>
     <sheet name="report1744993928915" sheetId="1" r:id="rId1"/>
@@ -3236,23 +3236,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFC9740D-89A1-4261-8CCB-623793D9C8FF}">
   <dimension ref="A1:M118"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.83203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="34.83203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="31.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="28.83203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="34.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="34.90625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.6328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.7265625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="31.6328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="28.90625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="34.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3293,7 +3293,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>13</v>
       </c>
@@ -3332,7 +3332,7 @@
       </c>
       <c r="M2" s="2"/>
     </row>
-    <row r="3" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" ht="58" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>22</v>
       </c>
@@ -3373,7 +3373,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>31</v>
       </c>
@@ -3412,7 +3412,7 @@
       </c>
       <c r="M4" s="2"/>
     </row>
-    <row r="5" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>39</v>
       </c>
@@ -3451,7 +3451,7 @@
       </c>
       <c r="M5" s="2"/>
     </row>
-    <row r="6" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" ht="58" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>48</v>
       </c>
@@ -3492,7 +3492,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>54</v>
       </c>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="M7" s="2"/>
     </row>
-    <row r="8" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>63</v>
       </c>
@@ -3570,7 +3570,7 @@
       </c>
       <c r="M8" s="2"/>
     </row>
-    <row r="9" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>69</v>
       </c>
@@ -3609,7 +3609,7 @@
       </c>
       <c r="M9" s="2"/>
     </row>
-    <row r="10" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" ht="58" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>77</v>
       </c>
@@ -3650,7 +3650,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>84</v>
       </c>
@@ -3689,7 +3689,7 @@
       </c>
       <c r="M11" s="2"/>
     </row>
-    <row r="12" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>92</v>
       </c>
@@ -3728,7 +3728,7 @@
       </c>
       <c r="M12" s="2"/>
     </row>
-    <row r="13" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>100</v>
       </c>
@@ -3767,7 +3767,7 @@
       </c>
       <c r="M13" s="2"/>
     </row>
-    <row r="14" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>105</v>
       </c>
@@ -3806,7 +3806,7 @@
       </c>
       <c r="M14" s="2"/>
     </row>
-    <row r="15" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>113</v>
       </c>
@@ -3845,7 +3845,7 @@
       </c>
       <c r="M15" s="2"/>
     </row>
-    <row r="16" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>121</v>
       </c>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="M16" s="2"/>
     </row>
-    <row r="17" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>129</v>
       </c>
@@ -3923,7 +3923,7 @@
       </c>
       <c r="M17" s="2"/>
     </row>
-    <row r="18" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>137</v>
       </c>
@@ -3962,7 +3962,7 @@
       </c>
       <c r="M18" s="2"/>
     </row>
-    <row r="19" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>144</v>
       </c>
@@ -4001,7 +4001,7 @@
       </c>
       <c r="M19" s="2"/>
     </row>
-    <row r="20" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>152</v>
       </c>
@@ -4040,7 +4040,7 @@
       </c>
       <c r="M20" s="2"/>
     </row>
-    <row r="21" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>158</v>
       </c>
@@ -4079,7 +4079,7 @@
       </c>
       <c r="M21" s="2"/>
     </row>
-    <row r="22" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>165</v>
       </c>
@@ -4118,7 +4118,7 @@
       </c>
       <c r="M22" s="2"/>
     </row>
-    <row r="23" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>173</v>
       </c>
@@ -4157,7 +4157,7 @@
       </c>
       <c r="M23" s="2"/>
     </row>
-    <row r="24" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>180</v>
       </c>
@@ -4196,7 +4196,7 @@
       </c>
       <c r="M24" s="2"/>
     </row>
-    <row r="25" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>188</v>
       </c>
@@ -4235,7 +4235,7 @@
       </c>
       <c r="M25" s="2"/>
     </row>
-    <row r="26" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>196</v>
       </c>
@@ -4274,7 +4274,7 @@
       </c>
       <c r="M26" s="2"/>
     </row>
-    <row r="27" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>204</v>
       </c>
@@ -4313,7 +4313,7 @@
       </c>
       <c r="M27" s="2"/>
     </row>
-    <row r="28" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>211</v>
       </c>
@@ -4352,7 +4352,7 @@
       </c>
       <c r="M28" s="2"/>
     </row>
-    <row r="29" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>219</v>
       </c>
@@ -4391,7 +4391,7 @@
       </c>
       <c r="M29" s="2"/>
     </row>
-    <row r="30" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:13" ht="58" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>221</v>
       </c>
@@ -4432,7 +4432,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="31" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>228</v>
       </c>
@@ -4471,7 +4471,7 @@
       </c>
       <c r="M31" s="2"/>
     </row>
-    <row r="32" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>236</v>
       </c>
@@ -4510,7 +4510,7 @@
       </c>
       <c r="M32" s="2"/>
     </row>
-    <row r="33" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>243</v>
       </c>
@@ -4549,7 +4549,7 @@
       </c>
       <c r="M33" s="2"/>
     </row>
-    <row r="34" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>251</v>
       </c>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="M34" s="2"/>
     </row>
-    <row r="35" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>259</v>
       </c>
@@ -4627,7 +4627,7 @@
       </c>
       <c r="M35" s="2"/>
     </row>
-    <row r="36" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>265</v>
       </c>
@@ -4666,7 +4666,7 @@
       </c>
       <c r="M36" s="2"/>
     </row>
-    <row r="37" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>273</v>
       </c>
@@ -4705,7 +4705,7 @@
       </c>
       <c r="M37" s="2"/>
     </row>
-    <row r="38" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>280</v>
       </c>
@@ -4744,7 +4744,7 @@
       </c>
       <c r="M38" s="2"/>
     </row>
-    <row r="39" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>288</v>
       </c>
@@ -4783,7 +4783,7 @@
       </c>
       <c r="M39" s="2"/>
     </row>
-    <row r="40" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>295</v>
       </c>
@@ -4822,7 +4822,7 @@
       </c>
       <c r="M40" s="2"/>
     </row>
-    <row r="41" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>303</v>
       </c>
@@ -4861,7 +4861,7 @@
       </c>
       <c r="M41" s="2"/>
     </row>
-    <row r="42" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>309</v>
       </c>
@@ -4900,7 +4900,7 @@
       </c>
       <c r="M42" s="2"/>
     </row>
-    <row r="43" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
         <v>315</v>
       </c>
@@ -4939,7 +4939,7 @@
       </c>
       <c r="M43" s="2"/>
     </row>
-    <row r="44" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
         <v>322</v>
       </c>
@@ -4978,7 +4978,7 @@
       </c>
       <c r="M44" s="2"/>
     </row>
-    <row r="45" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
         <v>330</v>
       </c>
@@ -5017,7 +5017,7 @@
       </c>
       <c r="M45" s="2"/>
     </row>
-    <row r="46" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
         <v>338</v>
       </c>
@@ -5056,7 +5056,7 @@
       </c>
       <c r="M46" s="2"/>
     </row>
-    <row r="47" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
         <v>345</v>
       </c>
@@ -5095,7 +5095,7 @@
       </c>
       <c r="M47" s="2"/>
     </row>
-    <row r="48" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
         <v>352</v>
       </c>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="M48" s="2"/>
     </row>
-    <row r="49" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
         <v>357</v>
       </c>
@@ -5165,7 +5165,7 @@
       </c>
       <c r="M49" s="2"/>
     </row>
-    <row r="50" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
         <v>365</v>
       </c>
@@ -5204,7 +5204,7 @@
       </c>
       <c r="M50" s="2"/>
     </row>
-    <row r="51" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
         <v>373</v>
       </c>
@@ -5235,7 +5235,7 @@
       </c>
       <c r="M51" s="2"/>
     </row>
-    <row r="52" spans="1:13" ht="32" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:13" ht="29" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
         <v>377</v>
       </c>
@@ -5274,7 +5274,7 @@
       </c>
       <c r="M52" s="2"/>
     </row>
-    <row r="53" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:13" ht="58" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
         <v>384</v>
       </c>
@@ -5315,7 +5315,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="54" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
         <v>392</v>
       </c>
@@ -5354,7 +5354,7 @@
       </c>
       <c r="M54" s="2"/>
     </row>
-    <row r="55" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:13" ht="58" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
         <v>398</v>
       </c>
@@ -5395,7 +5395,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="56" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
         <v>404</v>
       </c>
@@ -5434,7 +5434,7 @@
       </c>
       <c r="M56" s="2"/>
     </row>
-    <row r="57" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
         <v>412</v>
       </c>
@@ -5473,7 +5473,7 @@
       </c>
       <c r="M57" s="2"/>
     </row>
-    <row r="58" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:13" ht="58" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
         <v>419</v>
       </c>
@@ -5514,7 +5514,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="59" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
         <v>425</v>
       </c>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="M59" s="2"/>
     </row>
-    <row r="60" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>431</v>
       </c>
@@ -5592,7 +5592,7 @@
       </c>
       <c r="M60" s="2"/>
     </row>
-    <row r="61" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
         <v>438</v>
       </c>
@@ -5631,7 +5631,7 @@
       </c>
       <c r="M61" s="2"/>
     </row>
-    <row r="62" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:13" ht="58" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
         <v>445</v>
       </c>
@@ -5672,7 +5672,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="63" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A63" s="2" t="s">
         <v>452</v>
       </c>
@@ -5711,7 +5711,7 @@
       </c>
       <c r="M63" s="2"/>
     </row>
-    <row r="64" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A64" s="2" t="s">
         <v>457</v>
       </c>
@@ -5750,7 +5750,7 @@
       </c>
       <c r="M64" s="2"/>
     </row>
-    <row r="65" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:13" ht="58" x14ac:dyDescent="0.35">
       <c r="A65" s="2" t="s">
         <v>463</v>
       </c>
@@ -5791,7 +5791,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="66" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
         <v>470</v>
       </c>
@@ -5830,7 +5830,7 @@
       </c>
       <c r="M66" s="2"/>
     </row>
-    <row r="67" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:13" ht="58" x14ac:dyDescent="0.35">
       <c r="A67" s="2" t="s">
         <v>476</v>
       </c>
@@ -5871,7 +5871,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="68" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A68" s="2" t="s">
         <v>483</v>
       </c>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="M68" s="2"/>
     </row>
-    <row r="69" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A69" s="2" t="s">
         <v>490</v>
       </c>
@@ -5949,7 +5949,7 @@
       </c>
       <c r="M69" s="2"/>
     </row>
-    <row r="70" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A70" s="2" t="s">
         <v>498</v>
       </c>
@@ -5988,7 +5988,7 @@
       </c>
       <c r="M70" s="2"/>
     </row>
-    <row r="71" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A71" s="2" t="s">
         <v>500</v>
       </c>
@@ -6027,7 +6027,7 @@
       </c>
       <c r="M71" s="2"/>
     </row>
-    <row r="72" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A72" s="2" t="s">
         <v>508</v>
       </c>
@@ -6066,7 +6066,7 @@
       </c>
       <c r="M72" s="2"/>
     </row>
-    <row r="73" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A73" s="2" t="s">
         <v>516</v>
       </c>
@@ -6105,7 +6105,7 @@
       </c>
       <c r="M73" s="2"/>
     </row>
-    <row r="74" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:13" ht="29" x14ac:dyDescent="0.35">
       <c r="A74" s="2" t="s">
         <v>519</v>
       </c>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="M74" s="2"/>
     </row>
-    <row r="75" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A75" s="2" t="s">
         <v>524</v>
       </c>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="M75" s="2"/>
     </row>
-    <row r="76" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A76" s="2" t="s">
         <v>530</v>
       </c>
@@ -6222,7 +6222,7 @@
       </c>
       <c r="M76" s="2"/>
     </row>
-    <row r="77" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:13" ht="58" x14ac:dyDescent="0.35">
       <c r="A77" s="2" t="s">
         <v>536</v>
       </c>
@@ -6263,7 +6263,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="78" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A78" s="2" t="s">
         <v>542</v>
       </c>
@@ -6302,7 +6302,7 @@
       </c>
       <c r="M78" s="2"/>
     </row>
-    <row r="79" spans="1:13" ht="32" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:13" ht="29" x14ac:dyDescent="0.35">
       <c r="A79" s="2" t="s">
         <v>549</v>
       </c>
@@ -6341,7 +6341,7 @@
       </c>
       <c r="M79" s="2"/>
     </row>
-    <row r="80" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A80" s="2" t="s">
         <v>557</v>
       </c>
@@ -6380,7 +6380,7 @@
       </c>
       <c r="M80" s="2"/>
     </row>
-    <row r="81" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:13" ht="58" x14ac:dyDescent="0.35">
       <c r="A81" s="2" t="s">
         <v>563</v>
       </c>
@@ -6421,7 +6421,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="82" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:13" ht="58" x14ac:dyDescent="0.35">
       <c r="A82" s="2" t="s">
         <v>569</v>
       </c>
@@ -6462,7 +6462,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="83" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A83" s="2" t="s">
         <v>575</v>
       </c>
@@ -6501,7 +6501,7 @@
       </c>
       <c r="M83" s="2"/>
     </row>
-    <row r="84" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:13" ht="58" x14ac:dyDescent="0.35">
       <c r="A84" s="2" t="s">
         <v>583</v>
       </c>
@@ -6542,7 +6542,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="85" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:13" ht="58" x14ac:dyDescent="0.35">
       <c r="A85" s="2" t="s">
         <v>591</v>
       </c>
@@ -6583,7 +6583,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="86" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:13" ht="58" x14ac:dyDescent="0.35">
       <c r="A86" s="2" t="s">
         <v>598</v>
       </c>
@@ -6624,7 +6624,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="87" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A87" s="2" t="s">
         <v>605</v>
       </c>
@@ -6663,7 +6663,7 @@
       </c>
       <c r="M87" s="2"/>
     </row>
-    <row r="88" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A88" s="2" t="s">
         <v>606</v>
       </c>
@@ -6702,7 +6702,7 @@
       </c>
       <c r="M88" s="2"/>
     </row>
-    <row r="89" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A89" s="2" t="s">
         <v>614</v>
       </c>
@@ -6741,7 +6741,7 @@
       </c>
       <c r="M89" s="2"/>
     </row>
-    <row r="90" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:13" ht="58" x14ac:dyDescent="0.35">
       <c r="A90" s="2" t="s">
         <v>615</v>
       </c>
@@ -6782,7 +6782,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="91" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:13" ht="58" x14ac:dyDescent="0.35">
       <c r="A91" s="2" t="s">
         <v>622</v>
       </c>
@@ -6823,7 +6823,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="92" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:13" ht="58" x14ac:dyDescent="0.35">
       <c r="A92" s="2" t="s">
         <v>629</v>
       </c>
@@ -6864,7 +6864,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="93" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:13" ht="58" x14ac:dyDescent="0.35">
       <c r="A93" s="2" t="s">
         <v>631</v>
       </c>
@@ -6905,7 +6905,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="94" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A94" s="2" t="s">
         <v>634</v>
       </c>
@@ -6944,7 +6944,7 @@
       </c>
       <c r="M94" s="2"/>
     </row>
-    <row r="95" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:13" ht="58" x14ac:dyDescent="0.35">
       <c r="A95" s="2" t="s">
         <v>639</v>
       </c>
@@ -6985,7 +6985,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="96" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A96" s="2" t="s">
         <v>644</v>
       </c>
@@ -7024,7 +7024,7 @@
       </c>
       <c r="M96" s="2"/>
     </row>
-    <row r="97" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A97" s="2" t="s">
         <v>651</v>
       </c>
@@ -7063,7 +7063,7 @@
       </c>
       <c r="M97" s="2"/>
     </row>
-    <row r="98" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A98" s="2" t="s">
         <v>658</v>
       </c>
@@ -7102,7 +7102,7 @@
       </c>
       <c r="M98" s="2"/>
     </row>
-    <row r="99" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:13" ht="58" x14ac:dyDescent="0.35">
       <c r="A99" s="2" t="s">
         <v>666</v>
       </c>
@@ -7143,7 +7143,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="100" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A100" s="2" t="s">
         <v>667</v>
       </c>
@@ -7182,7 +7182,7 @@
       </c>
       <c r="M100" s="2"/>
     </row>
-    <row r="101" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A101" s="2" t="s">
         <v>673</v>
       </c>
@@ -7221,7 +7221,7 @@
       </c>
       <c r="M101" s="2"/>
     </row>
-    <row r="102" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:13" ht="58" x14ac:dyDescent="0.35">
       <c r="A102" s="2" t="s">
         <v>678</v>
       </c>
@@ -7262,7 +7262,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="103" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A103" s="2" t="s">
         <v>686</v>
       </c>
@@ -7301,7 +7301,7 @@
       </c>
       <c r="M103" s="2"/>
     </row>
-    <row r="104" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A104" s="2" t="s">
         <v>692</v>
       </c>
@@ -7340,7 +7340,7 @@
       </c>
       <c r="M104" s="2"/>
     </row>
-    <row r="105" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:13" ht="58" x14ac:dyDescent="0.35">
       <c r="A105" s="2" t="s">
         <v>698</v>
       </c>
@@ -7381,7 +7381,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="106" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A106" s="2" t="s">
         <v>704</v>
       </c>
@@ -7420,7 +7420,7 @@
       </c>
       <c r="M106" s="2"/>
     </row>
-    <row r="107" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:13" ht="58" x14ac:dyDescent="0.35">
       <c r="A107" s="2" t="s">
         <v>711</v>
       </c>
@@ -7461,7 +7461,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="108" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A108" s="2" t="s">
         <v>717</v>
       </c>
@@ -7500,7 +7500,7 @@
       </c>
       <c r="M108" s="2"/>
     </row>
-    <row r="109" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A109" s="2" t="s">
         <v>723</v>
       </c>
@@ -7539,7 +7539,7 @@
       </c>
       <c r="M109" s="2"/>
     </row>
-    <row r="110" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A110" s="2" t="s">
         <v>724</v>
       </c>
@@ -7578,7 +7578,7 @@
       </c>
       <c r="M110" s="2"/>
     </row>
-    <row r="111" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A111" s="2" t="s">
         <v>729</v>
       </c>
@@ -7617,7 +7617,7 @@
       </c>
       <c r="M111" s="2"/>
     </row>
-    <row r="112" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A112" s="2" t="s">
         <v>737</v>
       </c>
@@ -7656,7 +7656,7 @@
       </c>
       <c r="M112" s="2"/>
     </row>
-    <row r="113" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A113" s="2" t="s">
         <v>743</v>
       </c>
@@ -7695,7 +7695,7 @@
       </c>
       <c r="M113" s="2"/>
     </row>
-    <row r="114" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A114" s="2" t="s">
         <v>751</v>
       </c>
@@ -7734,7 +7734,7 @@
       </c>
       <c r="M114" s="2"/>
     </row>
-    <row r="115" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A115" s="2" t="s">
         <v>758</v>
       </c>
@@ -7773,7 +7773,7 @@
       </c>
       <c r="M115" s="2"/>
     </row>
-    <row r="116" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A116" s="2" t="s">
         <v>764</v>
       </c>
@@ -7812,7 +7812,7 @@
       </c>
       <c r="M116" s="2"/>
     </row>
-    <row r="117" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A117" s="2" t="s">
         <v>770</v>
       </c>
@@ -7851,7 +7851,7 @@
       </c>
       <c r="M117" s="2"/>
     </row>
-    <row r="118" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A118" s="2" t="s">
         <v>775</v>
       </c>

</xml_diff>